<commit_message>
Add renderer support for pillars.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8023281-1A43-4302-9472-7F3047DDEC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6F0CF1-D93C-4C5C-A89B-0CBC76F7D0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="21060" windowHeight="15585" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4411" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4369" uniqueCount="179">
   <si>
     <t>X</t>
   </si>
@@ -3695,7 +3695,7 @@
       <c r="AO3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AP3" s="2" t="s">
+      <c r="AP3" s="2">
         <v>0</v>
       </c>
       <c r="AQ3" s="2" t="s">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="BM3" s="1" t="str">
         <f t="shared" ref="BM3:BM64" si="0">_xlfn.TEXTJOIN("",TRUE,A3:BL3)</f>
-        <v>XXXXXXXXXXU|R#:*!BBSWWPPXXXAXBXXXSXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXU|R#:*!BBSWWPPXXXAXBXXXSXXXXXXX0XXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.25">
@@ -3887,19 +3887,19 @@
       <c r="AM4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR4" s="2" t="s">
+      <c r="AN4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR4" s="2">
         <v>0</v>
       </c>
       <c r="AS4" s="2" t="s">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="BM4" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXX00000000000000000000XXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXX00000000000000000000XXX0XXXXX00000XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="5" spans="1:65" x14ac:dyDescent="0.25">
@@ -4085,19 +4085,19 @@
       <c r="AM5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="2" t="s">
+      <c r="AN5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR5" s="2">
         <v>0</v>
       </c>
       <c r="AS5" s="2" t="s">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="BM5" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXX0E0F0XXXSXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXX0E0F0XXXSXXXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="6" spans="1:65" x14ac:dyDescent="0.25">
@@ -4283,19 +4283,19 @@
       <c r="AM6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR6" s="2" t="s">
+      <c r="AN6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="2">
         <v>0</v>
       </c>
       <c r="AS6" s="2" t="s">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="BM6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXX00000D00000D0A00XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXX00000D00000D0A00XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="7" spans="1:65" x14ac:dyDescent="0.25">
@@ -4481,19 +4481,19 @@
       <c r="AM7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AN7" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ7" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR7" s="2">
         <v>0</v>
       </c>
       <c r="AS7" s="2" t="s">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="BM7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XX10G02XXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX0XX10G02XXXX0XXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="8" spans="1:65" x14ac:dyDescent="0.25">
@@ -4679,19 +4679,19 @@
       <c r="AM8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR8" s="2" t="s">
+      <c r="AN8" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO8" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="2">
+        <v>0</v>
+      </c>
+      <c r="AQ8" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR8" s="2">
         <v>0</v>
       </c>
       <c r="AS8" s="2" t="s">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="BM8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXX0XXXXXXAXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXX0XXXXXXAXXXX00000XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="9" spans="1:65" x14ac:dyDescent="0.25">
@@ -4877,19 +4877,19 @@
       <c r="AM9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR9" s="2" t="s">
+      <c r="AN9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="2">
         <v>0</v>
       </c>
       <c r="AS9" s="2" t="s">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="BM9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXXDXXXXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXXDXXXXXX0XXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="10" spans="1:65" x14ac:dyDescent="0.25">
@@ -5075,19 +5075,19 @@
       <c r="AM10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR10" s="2" t="s">
+      <c r="AN10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AQ10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR10" s="2">
         <v>0</v>
       </c>
       <c r="AS10" s="2" t="s">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="BM10" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXAXXXX0XXXXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXAXXXX0XXXXXX0XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="11" spans="1:65" x14ac:dyDescent="0.25">
@@ -5273,19 +5273,19 @@
       <c r="AM11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR11" s="2" t="s">
+      <c r="AN11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP11" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR11" s="2">
         <v>0</v>
       </c>
       <c r="AS11" s="2" t="s">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="BM11" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000X000XXXXXAXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX000X000XXXXXAXXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="12" spans="1:65" x14ac:dyDescent="0.25">
@@ -5471,19 +5471,19 @@
       <c r="AM12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AR12" s="2" t="s">
+      <c r="AN12" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO12" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP12" s="2">
+        <v>0</v>
+      </c>
+      <c r="AQ12" s="2">
+        <v>0</v>
+      </c>
+      <c r="AR12" s="2">
         <v>0</v>
       </c>
       <c r="AS12" s="2" t="s">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="BM12" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0K0W0P0XXXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX0K0W0P0XXXXX0XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="13" spans="1:65" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add Menu system. Add objectives/briefs to map format.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6F0CF1-D93C-4C5C-A89B-0CBC76F7D0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97393C9-D8BD-40C7-A20A-32C41FAB20D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
@@ -2587,7 +2587,7 @@
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
         <v>24</v>
@@ -2613,7 +2613,7 @@
         <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F13" t="s">
         <v>24</v>
@@ -2639,7 +2639,7 @@
         <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F14" t="s">
         <v>24</v>
@@ -2665,7 +2665,7 @@
         <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F15" t="s">
         <v>24</v>
@@ -2743,7 +2743,7 @@
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F18" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
Add level event hooks.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97393C9-D8BD-40C7-A20A-32C41FAB20D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6833CB91-5610-44C2-8A02-77EC1AE21DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Optimisation" sheetId="7" r:id="rId8"/>
     <sheet name="Performance" sheetId="6" r:id="rId9"/>
     <sheet name="TIming" sheetId="11" r:id="rId10"/>
+    <sheet name="Cheats" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4369" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4301" uniqueCount="183">
   <si>
     <t>X</t>
   </si>
@@ -585,6 +586,18 @@
   </si>
   <si>
     <t>Item</t>
+  </si>
+  <si>
+    <t>Invincibility</t>
+  </si>
+  <si>
+    <t>All Weapons</t>
+  </si>
+  <si>
+    <t>Inifinite Ammo</t>
+  </si>
+  <si>
+    <t>? Decoration</t>
   </si>
 </sst>
 </file>
@@ -663,7 +676,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -688,6 +701,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2071,6 +2087,34 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBA98B54-E046-4741-B9FA-82889E746A76}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5235E873-4701-4130-881C-1F333236149A}">
   <dimension ref="A1:B5"/>
@@ -2284,6 +2328,11 @@
   <cols>
     <col min="1" max="1" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="2.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2943,7 +2992,7 @@
       <c r="G27" t="s">
         <v>24</v>
       </c>
-      <c r="M27">
+      <c r="M27" s="10">
         <v>1</v>
       </c>
     </row>
@@ -2969,7 +3018,7 @@
       <c r="G28" t="s">
         <v>24</v>
       </c>
-      <c r="M28">
+      <c r="M28" s="10">
         <v>2</v>
       </c>
     </row>
@@ -2995,7 +3044,7 @@
       <c r="G29" t="s">
         <v>24</v>
       </c>
-      <c r="M29">
+      <c r="M29" s="10">
         <v>3</v>
       </c>
     </row>
@@ -3021,7 +3070,7 @@
       <c r="G30" t="s">
         <v>24</v>
       </c>
-      <c r="M30">
+      <c r="M30" s="10">
         <v>4</v>
       </c>
     </row>
@@ -3047,7 +3096,7 @@
       <c r="G31" t="s">
         <v>24</v>
       </c>
-      <c r="M31">
+      <c r="M31" s="10">
         <v>5</v>
       </c>
     </row>
@@ -3073,44 +3122,204 @@
       <c r="G32" t="s">
         <v>24</v>
       </c>
-      <c r="M32">
+      <c r="M32" s="10">
         <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M33">
+      <c r="M33" s="10">
         <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34"/>
-      <c r="M34">
+      <c r="A34" s="14">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>173</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" t="s">
+        <v>24</v>
+      </c>
+      <c r="M34" s="10">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35"/>
+      <c r="A35" s="14">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>174</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" t="s">
+        <v>24</v>
+      </c>
       <c r="M35">
         <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36"/>
+      <c r="A36" s="14">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" t="s">
+        <v>24</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="37" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37"/>
+      <c r="A37" s="14">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" t="s">
+        <v>24</v>
+      </c>
+      <c r="F37" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="38" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38"/>
+      <c r="A38" s="14">
+        <v>5</v>
+      </c>
+      <c r="B38" t="s">
+        <v>182</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="39" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39"/>
+      <c r="A39" s="14">
+        <v>6</v>
+      </c>
+      <c r="B39" t="s">
+        <v>182</v>
+      </c>
+      <c r="C39" t="s">
+        <v>24</v>
+      </c>
+      <c r="D39" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" t="s">
+        <v>24</v>
+      </c>
+      <c r="F39" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="40" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40"/>
+      <c r="A40" s="14">
+        <v>7</v>
+      </c>
+      <c r="B40" t="s">
+        <v>182</v>
+      </c>
+      <c r="C40" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" t="s">
+        <v>24</v>
+      </c>
+      <c r="E40" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="41" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41"/>
+      <c r="A41" s="14">
+        <v>8</v>
+      </c>
+      <c r="B41" t="s">
+        <v>182</v>
+      </c>
+      <c r="C41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" t="s">
+        <v>24</v>
+      </c>
+      <c r="E41" t="s">
+        <v>24</v>
+      </c>
+      <c r="F41" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="42" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A42"/>
@@ -3401,103 +3610,103 @@
       <c r="I2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="2">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2">
-        <v>0</v>
-      </c>
-      <c r="P2" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>0</v>
-      </c>
-      <c r="R2" s="2">
-        <v>0</v>
-      </c>
-      <c r="S2" s="2">
-        <v>0</v>
-      </c>
-      <c r="T2" s="2">
-        <v>0</v>
-      </c>
-      <c r="U2" s="2">
-        <v>0</v>
-      </c>
-      <c r="V2" s="2">
-        <v>0</v>
-      </c>
-      <c r="W2" s="2">
-        <v>0</v>
-      </c>
-      <c r="X2" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="2">
+      <c r="AC2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AH2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AI2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AK2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AL2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AN2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AO2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AQ2" s="2" t="s">
@@ -3568,7 +3777,7 @@
       </c>
       <c r="BM2" s="1" t="str">
         <f>_xlfn.TEXTJOIN("",TRUE,A2:BL2)</f>
-        <v>XXXXXXXXXV000000000000000000000D0C00A00A00XXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXVXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="3" spans="1:65" x14ac:dyDescent="0.25">
@@ -3603,46 +3812,46 @@
         <v>0</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>165</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>163</v>
+        <v>0</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>159</v>
+        <v>0</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="2" t="s">
         <v>0</v>
@@ -3654,13 +3863,13 @@
         <v>0</v>
       </c>
       <c r="AB3" s="2" t="s">
-        <v>2</v>
+        <v>141</v>
       </c>
       <c r="AC3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD3" s="2" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="AE3" s="2" t="s">
         <v>0</v>
@@ -3672,7 +3881,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI3" s="2" t="s">
         <v>0</v>
@@ -3695,7 +3904,7 @@
       <c r="AO3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AP3" s="2">
+      <c r="AP3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AQ3" s="2" t="s">
@@ -3766,7 +3975,7 @@
       </c>
       <c r="BM3" s="1" t="str">
         <f t="shared" ref="BM3:BM64" si="0">_xlfn.TEXTJOIN("",TRUE,A3:BL3)</f>
-        <v>XXXXXXXXXXU|R#:*!BBSWWPPXXXAXBXXXSXXXXXXX0XXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXTXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.25">
@@ -3800,52 +4009,52 @@
       <c r="J4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="K4" s="2">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2">
-        <v>0</v>
-      </c>
-      <c r="O4" s="2">
-        <v>0</v>
-      </c>
-      <c r="P4" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="2">
-        <v>0</v>
-      </c>
-      <c r="R4" s="2">
-        <v>0</v>
-      </c>
-      <c r="S4" s="2">
-        <v>0</v>
-      </c>
-      <c r="T4" s="2">
-        <v>0</v>
-      </c>
-      <c r="U4" s="2">
-        <v>0</v>
-      </c>
-      <c r="V4" s="2">
-        <v>0</v>
-      </c>
-      <c r="W4" s="2">
-        <v>0</v>
-      </c>
-      <c r="X4" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="2">
+      <c r="K4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AA4" s="2">
@@ -3857,7 +4066,7 @@
       <c r="AC4" s="2">
         <v>0</v>
       </c>
-      <c r="AD4" s="2">
+      <c r="AD4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AE4" s="2" t="s">
@@ -3869,7 +4078,7 @@
       <c r="AG4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AH4" s="2">
+      <c r="AH4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AI4" s="2" t="s">
@@ -3887,19 +4096,19 @@
       <c r="AM4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AQ4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR4" s="2">
+      <c r="AN4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS4" s="2" t="s">
@@ -3964,7 +4173,7 @@
       </c>
       <c r="BM4" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXX00000000000000000000XXX0XXXXX00000XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXX000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="5" spans="1:65" x14ac:dyDescent="0.25">
@@ -4043,20 +4252,20 @@
       <c r="Y5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Z5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="2" t="s">
-        <v>58</v>
+      <c r="Z5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="2">
+        <v>0</v>
       </c>
       <c r="AB5" s="2">
         <v>0</v>
       </c>
-      <c r="AC5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AD5" s="2">
-        <v>0</v>
+      <c r="AC5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="AE5" s="2" t="s">
         <v>0</v>
@@ -4068,7 +4277,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI5" s="2" t="s">
         <v>0</v>
@@ -4085,19 +4294,19 @@
       <c r="AM5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP5" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ5" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="2">
+      <c r="AN5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS5" s="2" t="s">
@@ -4162,7 +4371,7 @@
       </c>
       <c r="BM5" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXX0E0F0XXXSXXXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXX000!XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="6" spans="1:65" x14ac:dyDescent="0.25">
@@ -4223,52 +4432,52 @@
       <c r="S6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="T6" s="2">
-        <v>0</v>
-      </c>
-      <c r="U6" s="2">
-        <v>0</v>
-      </c>
-      <c r="V6" s="2">
-        <v>0</v>
-      </c>
-      <c r="W6" s="2">
-        <v>0</v>
-      </c>
-      <c r="X6" s="2">
+      <c r="T6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Y6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="Z6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="2">
+      <c r="AC6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AE6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AG6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AH6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AJ6" s="2" t="s">
@@ -4283,19 +4492,19 @@
       <c r="AM6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AQ6" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR6" s="2">
+      <c r="AN6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS6" s="2" t="s">
@@ -4360,7 +4569,7 @@
       </c>
       <c r="BM6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXX00000D00000D0A00XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXDXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="7" spans="1:65" x14ac:dyDescent="0.25">
@@ -4430,7 +4639,7 @@
       <c r="V7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W7" s="2">
+      <c r="W7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="X7" s="2" t="s">
@@ -4439,20 +4648,20 @@
       <c r="Y7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Z7" s="2">
-        <v>1</v>
+      <c r="Z7" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="AA7" s="2">
         <v>0</v>
       </c>
-      <c r="AB7" s="2" t="s">
-        <v>60</v>
+      <c r="AB7" s="2">
+        <v>0</v>
       </c>
       <c r="AC7" s="2">
         <v>0</v>
       </c>
-      <c r="AD7" s="2">
-        <v>2</v>
+      <c r="AD7" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="AE7" s="2" t="s">
         <v>0</v>
@@ -4466,7 +4675,7 @@
       <c r="AH7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AI7" s="2">
+      <c r="AI7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AJ7" s="2" t="s">
@@ -4481,19 +4690,19 @@
       <c r="AM7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP7" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ7" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR7" s="2">
+      <c r="AN7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS7" s="2" t="s">
@@ -4558,7 +4767,7 @@
       </c>
       <c r="BM7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XX10G02XXXX0XXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXX000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="8" spans="1:65" x14ac:dyDescent="0.25">
@@ -4628,7 +4837,7 @@
       <c r="V8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W8" s="2">
+      <c r="W8" s="2" t="s">
         <v>0</v>
       </c>
       <c r="X8" s="2" t="s">
@@ -4640,14 +4849,14 @@
       <c r="Z8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AA8" s="2" t="s">
-        <v>0</v>
+      <c r="AA8" s="2">
+        <v>2</v>
       </c>
       <c r="AB8" s="2">
         <v>0</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>0</v>
+      <c r="AC8" s="2">
+        <v>1</v>
       </c>
       <c r="AD8" s="2" t="s">
         <v>0</v>
@@ -4665,7 +4874,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ8" s="2" t="s">
         <v>0</v>
@@ -4679,19 +4888,19 @@
       <c r="AM8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AQ8" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR8" s="2">
+      <c r="AN8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR8" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS8" s="2" t="s">
@@ -4756,7 +4965,7 @@
       </c>
       <c r="BM8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXX0XXXXXXAXXXX00000XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXX201XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="9" spans="1:65" x14ac:dyDescent="0.25">
@@ -4826,8 +5035,8 @@
       <c r="V9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W9" s="2">
-        <v>0</v>
+      <c r="W9" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="X9" s="2" t="s">
         <v>0</v>
@@ -4836,7 +5045,7 @@
         <v>0</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AA9" s="2" t="s">
         <v>0</v>
@@ -4862,7 +5071,7 @@
       <c r="AH9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AI9" s="2">
+      <c r="AI9" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AJ9" s="2" t="s">
@@ -4877,19 +5086,19 @@
       <c r="AM9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR9" s="2">
+      <c r="AN9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR9" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS9" s="2" t="s">
@@ -4954,7 +5163,7 @@
       </c>
       <c r="BM9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0XXXXDXXXXXX0XXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXX!XX!XDXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="10" spans="1:65" x14ac:dyDescent="0.25">
@@ -5021,19 +5230,19 @@
       <c r="U10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W10" s="2" t="s">
+      <c r="V10" s="2">
         <v>2</v>
       </c>
+      <c r="W10" s="2">
+        <v>0</v>
+      </c>
       <c r="X10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="2">
         <v>0</v>
       </c>
       <c r="AA10" s="2" t="s">
@@ -5045,22 +5254,22 @@
       <c r="AC10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AD10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE10" s="2" t="s">
+      <c r="AD10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="2">
         <v>0</v>
       </c>
       <c r="AF10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI10" s="2">
+        <v>1</v>
+      </c>
+      <c r="AG10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="2">
+        <v>2</v>
+      </c>
+      <c r="AI10" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AJ10" s="2" t="s">
@@ -5075,19 +5284,19 @@
       <c r="AM10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AQ10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR10" s="2">
+      <c r="AN10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR10" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS10" s="2" t="s">
@@ -5152,7 +5361,7 @@
       </c>
       <c r="BM10" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXAXXXX0XXXXXX0XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX20W00X0X00W02XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="11" spans="1:65" x14ac:dyDescent="0.25">
@@ -5217,49 +5426,49 @@
         <v>0</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="V11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="V11" s="2">
         <v>0</v>
       </c>
       <c r="W11" s="2">
         <v>0</v>
       </c>
-      <c r="X11" s="2">
+      <c r="X11" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Y11" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="2">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="Z11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="AB11" s="2">
         <v>0</v>
       </c>
-      <c r="AC11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE11" s="2" t="s">
-        <v>0</v>
+      <c r="AC11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="2">
+        <v>2</v>
       </c>
       <c r="AF11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AG11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="2" t="s">
+      <c r="AG11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="2">
         <v>0</v>
       </c>
       <c r="AI11" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ11" s="2" t="s">
         <v>0</v>
@@ -5273,19 +5482,19 @@
       <c r="AM11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP11" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="AQ11" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR11" s="2">
+      <c r="AN11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR11" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS11" s="2" t="s">
@@ -5350,7 +5559,7 @@
       </c>
       <c r="BM11" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000X000XXXXXAXXXX00|00XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXX!00X20D0D02X00XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="12" spans="1:65" x14ac:dyDescent="0.25">
@@ -5417,46 +5626,46 @@
       <c r="U12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W12" s="2">
-        <v>0</v>
+      <c r="V12" s="2">
+        <v>2</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>135</v>
+        <v>3</v>
       </c>
       <c r="Y12" s="2">
         <v>0</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AA12" s="2">
+        <v>45</v>
+      </c>
+      <c r="AA12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AB12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="AC12" s="2">
+        <v>2</v>
+      </c>
+      <c r="AC12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE12" s="2">
         <v>0</v>
       </c>
       <c r="AF12" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="2">
+        <v>45</v>
+      </c>
+      <c r="AH12" s="2">
+        <v>2</v>
+      </c>
+      <c r="AI12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AJ12" s="2" t="s">
@@ -5471,19 +5680,19 @@
       <c r="AM12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AN12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AO12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AP12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AQ12" s="2">
-        <v>0</v>
-      </c>
-      <c r="AR12" s="2">
+      <c r="AN12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AO12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AS12" s="2" t="s">
@@ -5548,7 +5757,7 @@
       </c>
       <c r="BM12" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX0K0W0P0XXXXX0XXXX00000XXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX2CD0CXAXC0DC2XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="13" spans="1:65" x14ac:dyDescent="0.25">
@@ -5613,49 +5822,49 @@
         <v>0</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="V13" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="V13" s="2">
         <v>0</v>
       </c>
       <c r="W13" s="2">
         <v>0</v>
       </c>
-      <c r="X13" s="2">
+      <c r="X13" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Y13" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="2">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="Z13" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="AB13" s="2">
         <v>0</v>
       </c>
-      <c r="AC13" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE13" s="2" t="s">
-        <v>0</v>
+      <c r="AC13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD13" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="2">
+        <v>2</v>
       </c>
       <c r="AF13" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AG13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="2">
-        <v>0</v>
+      <c r="AG13" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="AJ13" s="2" t="s">
         <v>0</v>
@@ -5746,7 +5955,7 @@
       </c>
       <c r="BM13" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000X000XXXXX0XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXX!00X20W0W02X00!XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="14" spans="1:65" x14ac:dyDescent="0.25">
@@ -5813,44 +6022,44 @@
       <c r="U14" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W14" s="2" t="s">
+      <c r="V14" s="2">
+        <v>2</v>
+      </c>
+      <c r="W14" s="2">
         <v>0</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="2">
         <v>0</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AB14" s="2" t="s">
+      <c r="AB14" s="2">
         <v>0</v>
       </c>
       <c r="AC14" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AD14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="2" t="s">
+      <c r="AD14" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="2">
         <v>0</v>
       </c>
       <c r="AF14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AG14" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="2">
+        <v>2</v>
       </c>
       <c r="AI14" s="2" t="s">
         <v>0</v>
@@ -5944,7 +6153,7 @@
       </c>
       <c r="BM14" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXTXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX20W00X0X00W02XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="15" spans="1:65" x14ac:dyDescent="0.25">
@@ -6014,13 +6223,13 @@
       <c r="V15" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="W15" s="2">
-        <v>0</v>
-      </c>
-      <c r="X15" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="2">
+      <c r="W15" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X15" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Z15" s="2" t="s">
@@ -6030,13 +6239,13 @@
         <v>0</v>
       </c>
       <c r="AB15" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC15" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD15" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AE15" s="2" t="s">
         <v>0</v>
@@ -6142,7 +6351,7 @@
       </c>
       <c r="BM15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXDX!XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="16" spans="1:65" x14ac:dyDescent="0.25">
@@ -6207,46 +6416,46 @@
         <v>0</v>
       </c>
       <c r="U16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="V16" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
+      </c>
+      <c r="V16" s="2">
+        <v>2</v>
       </c>
       <c r="W16" s="2">
         <v>0</v>
       </c>
-      <c r="X16" s="2">
-        <v>0</v>
+      <c r="X16" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="Y16" s="2">
         <v>0</v>
       </c>
-      <c r="Z16" s="2" t="s">
+      <c r="Z16" s="2">
         <v>0</v>
       </c>
       <c r="AA16" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AB16" s="2" t="s">
+      <c r="AB16" s="2">
         <v>0</v>
       </c>
       <c r="AC16" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AD16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="2" t="s">
+      <c r="AD16" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="2">
         <v>0</v>
       </c>
       <c r="AF16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AG16" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="2">
+        <v>2</v>
       </c>
       <c r="AI16" s="2" t="s">
         <v>0</v>
@@ -6340,7 +6549,7 @@
       </c>
       <c r="BM16" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXX!20W00X0X00W02XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="17" spans="1:65" x14ac:dyDescent="0.25">
@@ -6407,43 +6616,43 @@
       <c r="U17" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V17" s="2" t="s">
+      <c r="V17" s="2">
         <v>0</v>
       </c>
       <c r="W17" s="2">
         <v>0</v>
       </c>
-      <c r="X17" s="2">
+      <c r="X17" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Y17" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Z17" s="2">
         <v>0</v>
       </c>
       <c r="AA17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="2">
         <v>0</v>
       </c>
       <c r="AC17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE17" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AD17" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="2">
+        <v>2</v>
       </c>
       <c r="AF17" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AG17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH17" s="2" t="s">
+      <c r="AG17" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="2">
         <v>0</v>
       </c>
       <c r="AI17" s="2" t="s">
@@ -6538,7 +6747,7 @@
       </c>
       <c r="BM17" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXX000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX00X20D0D02X00XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="18" spans="1:65" x14ac:dyDescent="0.25">
@@ -6605,47 +6814,47 @@
       <c r="U18" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V18" s="2" t="s">
-        <v>0</v>
+      <c r="V18" s="2">
+        <v>2</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="X18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y18" s="2">
         <v>0</v>
       </c>
       <c r="Z18" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="AA18" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AB18" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC18" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE18" s="2">
         <v>0</v>
       </c>
       <c r="AF18" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="AH18" s="2">
+        <v>2</v>
       </c>
       <c r="AI18" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AJ18" s="2" t="s">
         <v>0</v>
@@ -6736,7 +6945,7 @@
       </c>
       <c r="BM18" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX2CD0CXAXC0DC2!XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="19" spans="1:65" x14ac:dyDescent="0.25">
@@ -6803,43 +7012,43 @@
       <c r="U19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="V19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W19" s="2" t="s">
+      <c r="V19" s="2">
+        <v>0</v>
+      </c>
+      <c r="W19" s="2">
         <v>0</v>
       </c>
       <c r="X19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="2" t="s">
+      <c r="Y19" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z19" s="2">
         <v>0</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="2">
         <v>0</v>
       </c>
       <c r="AC19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE19" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="2">
+        <v>2</v>
       </c>
       <c r="AF19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AG19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH19" s="2" t="s">
+      <c r="AG19" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="2">
         <v>0</v>
       </c>
       <c r="AI19" s="2" t="s">
@@ -6934,7 +7143,7 @@
       </c>
       <c r="BM19" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX00X20W0W02X00XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="20" spans="1:65" x14ac:dyDescent="0.25">
@@ -7002,43 +7211,43 @@
         <v>0</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W20" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="W20" s="2">
         <v>0</v>
       </c>
       <c r="X20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="2">
         <v>0</v>
       </c>
       <c r="AA20" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AB20" s="2" t="s">
+      <c r="AB20" s="2">
         <v>0</v>
       </c>
       <c r="AC20" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AD20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="2" t="s">
+      <c r="AD20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="2">
         <v>0</v>
       </c>
       <c r="AF20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH20" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AG20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="2">
+        <v>2</v>
       </c>
       <c r="AI20" s="2" t="s">
         <v>0</v>
@@ -7132,7 +7341,7 @@
       </c>
       <c r="BM20" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXK0W00X0X00W02XXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="21" spans="1:65" x14ac:dyDescent="0.25">
@@ -7200,7 +7409,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>0</v>
@@ -7212,12 +7421,12 @@
         <v>0</v>
       </c>
       <c r="Z21" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AA21" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AB21" s="2">
         <v>0</v>
       </c>
       <c r="AC21" s="2" t="s">
@@ -7330,7 +7539,7 @@
       </c>
       <c r="BM21" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX!XXX!!0XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="22" spans="1:65" x14ac:dyDescent="0.25">
@@ -7415,29 +7624,29 @@
       <c r="AA22" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="AB22" s="2" t="s">
+      <c r="AB22" s="2">
         <v>0</v>
       </c>
       <c r="AC22" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AE22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AF22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AG22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AH22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AI22" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AJ22" s="2" t="s">
         <v>0</v>
@@ -7528,7 +7737,7 @@
       </c>
       <c r="BM22" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXX0X######XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="23" spans="1:65" x14ac:dyDescent="0.25">
@@ -7565,31 +7774,31 @@
       <c r="K23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O23" s="2" t="s">
+      <c r="L23" s="2">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2">
+        <v>0</v>
+      </c>
+      <c r="N23" s="2">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2">
         <v>0</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T23" s="2" t="s">
+      <c r="Q23" s="2">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2">
+        <v>0</v>
+      </c>
+      <c r="T23" s="2">
         <v>0</v>
       </c>
       <c r="U23" s="2" t="s">
@@ -7604,41 +7813,41 @@
       <c r="X23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y23" s="2" t="s">
+      <c r="Y23" s="2">
         <v>0</v>
       </c>
       <c r="Z23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="AA23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="2">
         <v>0</v>
       </c>
       <c r="AD23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="2">
         <v>0</v>
       </c>
       <c r="AJ23" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AK23" s="2" t="s">
         <v>0</v>
@@ -7726,7 +7935,7 @@
       </c>
       <c r="BM23" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000X0000XXXX0T000D00000#XXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="24" spans="1:65" x14ac:dyDescent="0.25">
@@ -7763,31 +7972,31 @@
       <c r="K24" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L24" s="2" t="s">
+      <c r="L24" s="2">
         <v>0</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="O24" s="2">
         <v>0</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R24" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2">
         <v>0</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T24" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T24" s="2">
         <v>0</v>
       </c>
       <c r="U24" s="2" t="s">
@@ -7803,37 +8012,37 @@
         <v>0</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AA24" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AB24" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AC24" s="2" t="s">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AD24" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AE24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF24" s="2">
         <v>0</v>
       </c>
       <c r="AG24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH24" s="2">
         <v>0</v>
       </c>
       <c r="AI24" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ24" s="2" t="s">
         <v>0</v>
@@ -7924,7 +8133,7 @@
       </c>
       <c r="BM24" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0|C0D00|0XXXXAX!X!#P0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="25" spans="1:65" x14ac:dyDescent="0.25">
@@ -7961,31 +8170,31 @@
       <c r="K25" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O25" s="2" t="s">
+      <c r="L25" s="2">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2">
+        <v>0</v>
+      </c>
+      <c r="N25" s="2">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2">
         <v>0</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R25" s="2">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2">
+        <v>0</v>
+      </c>
+      <c r="T25" s="2">
         <v>0</v>
       </c>
       <c r="U25" s="2" t="s">
@@ -8000,7 +8209,7 @@
       <c r="X25" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y25" s="2" t="s">
+      <c r="Y25" s="2">
         <v>0</v>
       </c>
       <c r="Z25" s="2" t="s">
@@ -8019,19 +8228,19 @@
         <v>0</v>
       </c>
       <c r="AE25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF25" s="2">
         <v>0</v>
       </c>
       <c r="AG25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH25" s="2">
         <v>0</v>
       </c>
       <c r="AI25" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ25" s="2" t="s">
         <v>0</v>
@@ -8122,7 +8331,7 @@
       </c>
       <c r="BM25" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000XC000XXXX0XXXXXP0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="26" spans="1:65" x14ac:dyDescent="0.25">
@@ -8159,31 +8368,31 @@
       <c r="K26" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O26" s="2" t="s">
+      <c r="L26" s="2">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2">
+        <v>0</v>
+      </c>
+      <c r="N26" s="2">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2">
         <v>0</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2">
+        <v>0</v>
+      </c>
+      <c r="T26" s="2">
         <v>0</v>
       </c>
       <c r="U26" s="2" t="s">
@@ -8196,19 +8405,19 @@
         <v>0</v>
       </c>
       <c r="X26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y26" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y26" s="2">
         <v>0</v>
       </c>
       <c r="Z26" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AA26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="2" t="s">
-        <v>0</v>
+        <v>58</v>
+      </c>
+      <c r="AB26" s="2">
+        <v>2</v>
       </c>
       <c r="AC26" s="2" t="s">
         <v>0</v>
@@ -8217,19 +8426,19 @@
         <v>0</v>
       </c>
       <c r="AE26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF26" s="2">
         <v>0</v>
       </c>
       <c r="AG26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH26" s="2">
         <v>0</v>
       </c>
       <c r="AI26" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ26" s="2" t="s">
         <v>0</v>
@@ -8320,7 +8529,7 @@
       </c>
       <c r="BM26" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000B0000XXXE0XE2XXP0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="27" spans="1:65" x14ac:dyDescent="0.25">
@@ -8358,79 +8567,79 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O27" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N27" s="2">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2">
         <v>0</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="Q27" s="2">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2">
         <v>0</v>
       </c>
       <c r="S27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T27" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T27" s="2">
         <v>0</v>
       </c>
       <c r="U27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="V27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="V27" s="2">
         <v>0</v>
       </c>
       <c r="W27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="X27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="X27" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="2">
         <v>0</v>
       </c>
       <c r="Z27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="2">
         <v>0</v>
       </c>
       <c r="AC27" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AD27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI27" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI27" s="2">
         <v>0</v>
       </c>
       <c r="AJ27" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AK27" s="2" t="s">
         <v>0</v>
@@ -8518,7 +8727,7 @@
       </c>
       <c r="BM27" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXC|00X00|0D0D00D00X#00000#XXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="28" spans="1:65" x14ac:dyDescent="0.25">
@@ -8555,31 +8764,31 @@
       <c r="K28" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O28" s="2" t="s">
+      <c r="L28" s="2">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2">
+        <v>0</v>
+      </c>
+      <c r="N28" s="2">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2">
         <v>0</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>0</v>
+      </c>
+      <c r="R28" s="2">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2">
+        <v>0</v>
+      </c>
+      <c r="T28" s="2">
         <v>0</v>
       </c>
       <c r="U28" s="2" t="s">
@@ -8592,19 +8801,19 @@
         <v>0</v>
       </c>
       <c r="X28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y28" s="2">
         <v>0</v>
       </c>
       <c r="Z28" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AA28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB28" s="2" t="s">
-        <v>0</v>
+        <v>58</v>
+      </c>
+      <c r="AB28" s="2">
+        <v>2</v>
       </c>
       <c r="AC28" s="2" t="s">
         <v>0</v>
@@ -8613,19 +8822,19 @@
         <v>0</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF28" s="2">
         <v>0</v>
       </c>
       <c r="AG28" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH28" s="2">
         <v>0</v>
       </c>
       <c r="AI28" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ28" s="2" t="s">
         <v>0</v>
@@ -8716,7 +8925,7 @@
       </c>
       <c r="BM28" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000B0000XXXE0XE2XXP0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="29" spans="1:65" x14ac:dyDescent="0.25">
@@ -8753,32 +8962,32 @@
       <c r="K29" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O29" s="2" t="s">
+      <c r="L29" s="2">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2">
+        <v>0</v>
+      </c>
+      <c r="N29" s="2">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2">
         <v>0</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S29" s="2" t="s">
+      <c r="Q29" s="2">
+        <v>0</v>
+      </c>
+      <c r="R29" s="2">
+        <v>0</v>
+      </c>
+      <c r="S29" s="2">
         <v>0</v>
       </c>
       <c r="T29" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="U29" s="2" t="s">
         <v>0</v>
@@ -8792,7 +9001,7 @@
       <c r="X29" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y29" s="2" t="s">
+      <c r="Y29" s="2">
         <v>0</v>
       </c>
       <c r="Z29" s="2" t="s">
@@ -8811,19 +9020,19 @@
         <v>0</v>
       </c>
       <c r="AE29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF29" s="2">
         <v>0</v>
       </c>
       <c r="AG29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH29" s="2">
         <v>0</v>
       </c>
       <c r="AI29" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ29" s="2" t="s">
         <v>0</v>
@@ -8914,7 +9123,7 @@
       </c>
       <c r="BM29" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000X000CXXXX0XXXXXP0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="30" spans="1:65" x14ac:dyDescent="0.25">
@@ -8951,31 +9160,31 @@
       <c r="K30" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="L30" s="2">
         <v>0</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N30" s="2">
         <v>0</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R30" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R30" s="2">
         <v>0</v>
       </c>
       <c r="S30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T30" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T30" s="2">
         <v>0</v>
       </c>
       <c r="U30" s="2" t="s">
@@ -8991,37 +9200,37 @@
         <v>0</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>0</v>
       </c>
       <c r="AA30" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AB30" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AC30" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AD30" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AE30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF30" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF30" s="2">
         <v>0</v>
       </c>
       <c r="AG30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH30" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH30" s="2">
         <v>0</v>
       </c>
       <c r="AI30" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AJ30" s="2" t="s">
         <v>0</v>
@@ -9112,7 +9321,7 @@
       </c>
       <c r="BM30" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0|0CDC0|0XXXXAX::::P0P0PXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="31" spans="1:65" x14ac:dyDescent="0.25">
@@ -9149,31 +9358,31 @@
       <c r="K31" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O31" s="2" t="s">
+      <c r="L31" s="2">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2">
         <v>0</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T31" s="2" t="s">
+      <c r="Q31" s="2">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2">
+        <v>0</v>
+      </c>
+      <c r="S31" s="2">
+        <v>0</v>
+      </c>
+      <c r="T31" s="2">
         <v>0</v>
       </c>
       <c r="U31" s="2" t="s">
@@ -9188,41 +9397,41 @@
       <c r="X31" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y31" s="2" t="s">
+      <c r="Y31" s="2">
         <v>0</v>
       </c>
       <c r="Z31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AC31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="2">
         <v>0</v>
       </c>
       <c r="AD31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AE31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AE31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="2">
         <v>0</v>
       </c>
       <c r="AJ31" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AK31" s="2" t="s">
         <v>0</v>
@@ -9310,7 +9519,7 @@
       </c>
       <c r="BM31" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000X0000XXXX0S000S00000#XXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="32" spans="1:65" x14ac:dyDescent="0.25">
@@ -9354,7 +9563,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>0</v>
@@ -9366,7 +9575,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S32" s="2" t="s">
         <v>0</v>
@@ -9393,34 +9602,34 @@
         <v>0</v>
       </c>
       <c r="AA32" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AB32" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AC32" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AD32" s="2" t="s">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AE32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AH32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI32" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF32" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG32" s="2">
+        <v>0</v>
+      </c>
+      <c r="AH32" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI32" s="2">
         <v>0</v>
       </c>
       <c r="AJ32" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AK32" s="2" t="s">
         <v>0</v>
@@ -9508,7 +9717,7 @@
       </c>
       <c r="BM32" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXDXXXDXXXXXXXX::::#0000#XXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="33" spans="1:65" x14ac:dyDescent="0.25">
@@ -9545,31 +9754,31 @@
       <c r="K33" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O33" s="2" t="s">
+      <c r="L33" s="2">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2">
         <v>0</v>
       </c>
       <c r="P33" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T33" s="2" t="s">
+      <c r="Q33" s="2">
+        <v>0</v>
+      </c>
+      <c r="R33" s="2">
+        <v>0</v>
+      </c>
+      <c r="S33" s="2">
+        <v>0</v>
+      </c>
+      <c r="T33" s="2">
         <v>0</v>
       </c>
       <c r="U33" s="2" t="s">
@@ -9606,16 +9815,16 @@
         <v>0</v>
       </c>
       <c r="AF33" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AG33" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AH33" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AI33" s="2" t="s">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="AJ33" s="2" t="s">
         <v>0</v>
@@ -9706,7 +9915,7 @@
       </c>
       <c r="BM33" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000X0000XXXXXXXXXXX####XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="34" spans="1:65" x14ac:dyDescent="0.25">
@@ -9743,31 +9952,31 @@
       <c r="K34" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" s="2">
         <v>0</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N34" s="2">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2">
         <v>0</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2">
         <v>0</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T34" s="2">
         <v>0</v>
       </c>
       <c r="U34" s="2" t="s">
@@ -9904,7 +10113,7 @@
       </c>
       <c r="BM34" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0|00D00|0XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="35" spans="1:65" x14ac:dyDescent="0.25">
@@ -9941,31 +10150,31 @@
       <c r="K35" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M35" s="2" t="s">
+      <c r="L35" s="2">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2">
         <v>0</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O35" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="O35" s="2">
         <v>0</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T35" s="2" t="s">
+      <c r="Q35" s="2">
+        <v>0</v>
+      </c>
+      <c r="R35" s="2">
+        <v>0</v>
+      </c>
+      <c r="S35" s="2">
+        <v>0</v>
+      </c>
+      <c r="T35" s="2">
         <v>0</v>
       </c>
       <c r="U35" s="2" t="s">
@@ -10102,7 +10311,7 @@
       </c>
       <c r="BM35" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX00C0X0000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="36" spans="1:65" x14ac:dyDescent="0.25">
@@ -10139,31 +10348,31 @@
       <c r="K36" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O36" s="2" t="s">
+      <c r="L36" s="2">
+        <v>0</v>
+      </c>
+      <c r="M36" s="2">
+        <v>0</v>
+      </c>
+      <c r="N36" s="2">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2">
         <v>0</v>
       </c>
       <c r="P36" s="2" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="Q36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T36" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R36" s="2">
+        <v>0</v>
+      </c>
+      <c r="S36" s="2">
+        <v>0</v>
+      </c>
+      <c r="T36" s="2">
         <v>0</v>
       </c>
       <c r="U36" s="2" t="s">
@@ -10300,7 +10509,7 @@
       </c>
       <c r="BM36" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000BC000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="37" spans="1:65" x14ac:dyDescent="0.25">
@@ -10337,31 +10546,31 @@
       <c r="K37" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="L37" s="2">
         <v>0</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O37" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N37" s="2">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2">
         <v>0</v>
       </c>
       <c r="P37" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q37" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R37" s="2" t="s">
+      <c r="Q37" s="2">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2">
         <v>0</v>
       </c>
       <c r="S37" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T37" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T37" s="2">
         <v>0</v>
       </c>
       <c r="U37" s="2" t="s">
@@ -10498,7 +10707,7 @@
       </c>
       <c r="BM37" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0|00X00|0XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="38" spans="1:65" x14ac:dyDescent="0.25">
@@ -10535,32 +10744,32 @@
       <c r="K38" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O38" s="2" t="s">
+      <c r="L38" s="2">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0</v>
+      </c>
+      <c r="N38" s="2">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2">
         <v>0</v>
       </c>
       <c r="P38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>0</v>
+      </c>
+      <c r="R38" s="2">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2">
         <v>0</v>
       </c>
       <c r="T38" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="U38" s="2" t="s">
         <v>0</v>
@@ -10696,7 +10905,7 @@
       </c>
       <c r="BM38" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000B000CXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="39" spans="1:65" x14ac:dyDescent="0.25">
@@ -10733,31 +10942,31 @@
       <c r="K39" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M39" s="2" t="s">
+      <c r="L39" s="2">
+        <v>0</v>
+      </c>
+      <c r="M39" s="2">
         <v>0</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O39" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="O39" s="2">
         <v>0</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T39" s="2" t="s">
+      <c r="Q39" s="2">
+        <v>0</v>
+      </c>
+      <c r="R39" s="2">
+        <v>0</v>
+      </c>
+      <c r="S39" s="2">
+        <v>0</v>
+      </c>
+      <c r="T39" s="2">
         <v>0</v>
       </c>
       <c r="U39" s="2" t="s">
@@ -10894,7 +11103,7 @@
       </c>
       <c r="BM39" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX00C0X0000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="40" spans="1:65" x14ac:dyDescent="0.25">
@@ -10931,31 +11140,31 @@
       <c r="K40" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L40" s="2" t="s">
+      <c r="L40" s="2">
         <v>0</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N40" s="2">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2">
         <v>0</v>
       </c>
       <c r="P40" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R40" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>0</v>
+      </c>
+      <c r="R40" s="2">
         <v>0</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="T40" s="2">
         <v>0</v>
       </c>
       <c r="U40" s="2" t="s">
@@ -11092,7 +11301,7 @@
       </c>
       <c r="BM40" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0|00D00|0XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="41" spans="1:65" x14ac:dyDescent="0.25">
@@ -11129,31 +11338,31 @@
       <c r="K41" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O41" s="2" t="s">
+      <c r="L41" s="2">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2">
+        <v>0</v>
+      </c>
+      <c r="N41" s="2">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2">
         <v>0</v>
       </c>
       <c r="P41" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Q41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="T41" s="2" t="s">
+      <c r="Q41" s="2">
+        <v>0</v>
+      </c>
+      <c r="R41" s="2">
+        <v>0</v>
+      </c>
+      <c r="S41" s="2">
+        <v>0</v>
+      </c>
+      <c r="T41" s="2">
         <v>0</v>
       </c>
       <c r="U41" s="2" t="s">
@@ -11290,7 +11499,7 @@
       </c>
       <c r="BM41" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXX0000X0000XXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="42" spans="1:65" x14ac:dyDescent="0.25">
@@ -15848,12 +16057,12 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:BL64">
+  <conditionalFormatting sqref="AD31:BL31 X31:AB31 A1:BL22 X32:BL32 A23:W32 A33:BL64 X23:BL30">
     <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="X">
       <formula>NOT(ISERROR(SEARCH("X",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:BL1048576">
+  <conditionalFormatting sqref="AD31:BL31 X31:AB31 A1:BL22 X32:BL32 A23:W32 A33:BL1048576 X23:BL30">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"D"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Sound files and docs.
</commit_message>
<xml_diff>
--- a/Psion Levels.xlsx
+++ b/Psion Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zak\Documents\GitProjects\psion3d\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590F8C16-D3B1-458B-98E4-7377A767816D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93771E32-F270-4C68-B21B-DE967CEB5D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="10" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{72A343FB-71F0-4738-BBFF-B23B40D170FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapbits" sheetId="4" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4300" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4298" uniqueCount="197">
   <si>
     <t>X</t>
   </si>
@@ -6924,8 +6924,8 @@
       <c r="V18" s="2">
         <v>2</v>
       </c>
-      <c r="W18" s="2" t="s">
-        <v>45</v>
+      <c r="W18" s="2">
+        <v>0</v>
       </c>
       <c r="X18" s="2" t="s">
         <v>3</v>
@@ -6933,8 +6933,8 @@
       <c r="Y18" s="2">
         <v>0</v>
       </c>
-      <c r="Z18" s="2" t="s">
-        <v>45</v>
+      <c r="Z18" s="2">
+        <v>0</v>
       </c>
       <c r="AA18" s="2" t="s">
         <v>0</v>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="BM18" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>XXXXXXXXXXXXXXXXXXXXX2CD0CXAXC0DC2!XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
+        <v>XXXXXXXXXXXXXXXXXXXXX20D00XAXC0DC2!XXXXXXXXXXXXXXXXXXXXXXXXXXXXX</v>
       </c>
     </row>
     <row r="19" spans="1:65" x14ac:dyDescent="0.25">

</xml_diff>